<commit_message>
atualizacao dos dados do 2Q26 da INTC
</commit_message>
<xml_diff>
--- a/analise_eua/semicondutores/intel/intc_indicators.xlsx
+++ b/analise_eua/semicondutores/intel/intc_indicators.xlsx
@@ -1453,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1610,88 +1610,88 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46109</v>
+        <v>46200</v>
       </c>
       <c r="B2" t="n">
-        <v>-60.17</v>
+        <v>-64.59</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>-1.56</v>
+        <v>-1.91</v>
       </c>
       <c r="E2" t="n">
-        <v>-234</v>
+        <v>4785</v>
       </c>
       <c r="F2" t="n">
-        <v>-27.46</v>
+        <v>-68.41</v>
       </c>
       <c r="G2" t="n">
-        <v>2.01</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>224312790</v>
+        <v>712671520</v>
       </c>
       <c r="I2" t="n">
-        <v>55462</v>
+        <v>65614</v>
       </c>
       <c r="J2" t="n">
-        <v>15542</v>
+        <v>16853</v>
       </c>
       <c r="K2" t="n">
-        <v>39920</v>
+        <v>48761</v>
       </c>
       <c r="L2" t="n">
-        <v>8.08</v>
+        <v>6.41</v>
       </c>
       <c r="M2" t="n">
-        <v>0.36</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>53.46</v>
+        <v>100.14</v>
       </c>
       <c r="O2" t="n">
-        <v>-3.06</v>
+        <v>-15.55</v>
       </c>
       <c r="P2" t="n">
-        <v>-4.27</v>
+        <v>-3.11</v>
       </c>
       <c r="Q2" t="n">
-        <v>1096</v>
+        <v>7006</v>
       </c>
       <c r="R2" t="n">
-        <v>3093</v>
+        <v>-3762</v>
       </c>
       <c r="S2" t="n">
-        <v>-1206</v>
+        <v>-7342</v>
       </c>
       <c r="T2" t="n">
-        <v>-2540</v>
+        <v>4450</v>
       </c>
       <c r="U2" t="n">
-        <v>3636</v>
+        <v>2556</v>
       </c>
       <c r="V2" t="n">
-        <v>3921</v>
+        <v>730</v>
       </c>
       <c r="W2" t="n">
-        <v>3375</v>
+        <v>3368</v>
       </c>
       <c r="X2" t="n">
-        <v>17851</v>
+        <v>14388</v>
       </c>
       <c r="Y2" t="n">
-        <v>35272</v>
+        <v>21543</v>
       </c>
       <c r="Z2" t="n">
-        <v>-299.64</v>
+        <v>-276.72</v>
       </c>
       <c r="AA2" t="n">
-        <v>-16073</v>
+        <v>-13697</v>
       </c>
       <c r="AB2" t="n">
-        <v>-13852</v>
+        <v>-3346</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -1705,94 +1705,94 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45927</v>
+        <v>46109</v>
       </c>
       <c r="B3" t="n">
-        <v>37.27</v>
+        <v>-60.17</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>-11.45</v>
+        <v>-1.56</v>
       </c>
       <c r="E3" t="n">
-        <v>3441</v>
+        <v>-234</v>
       </c>
       <c r="F3" t="n">
-        <v>29.76</v>
+        <v>-27.46</v>
       </c>
       <c r="G3" t="n">
-        <v>1.42</v>
+        <v>2.01</v>
       </c>
       <c r="H3" t="n">
-        <v>151444700</v>
+        <v>224312790</v>
       </c>
       <c r="I3" t="n">
-        <v>57983</v>
+        <v>55462</v>
       </c>
       <c r="J3" t="n">
-        <v>19794</v>
+        <v>15542</v>
       </c>
       <c r="K3" t="n">
-        <v>38189</v>
+        <v>39920</v>
       </c>
       <c r="L3" t="n">
-        <v>-60.43</v>
+        <v>8.08</v>
       </c>
       <c r="M3" t="n">
         <v>0.36</v>
       </c>
       <c r="N3" t="n">
-        <v>-300.05</v>
+        <v>53.46</v>
       </c>
       <c r="O3" t="n">
-        <v>-15.34</v>
+        <v>-3.06</v>
       </c>
       <c r="P3" t="n">
-        <v>-12.54</v>
+        <v>-4.27</v>
       </c>
       <c r="Q3" t="n">
-        <v>2546</v>
+        <v>1096</v>
       </c>
       <c r="R3" t="n">
-        <v>-6250</v>
+        <v>3093</v>
       </c>
       <c r="S3" t="n">
-        <v>5152</v>
+        <v>-1206</v>
       </c>
       <c r="T3" t="n">
-        <v>121</v>
+        <v>-2540</v>
       </c>
       <c r="U3" t="n">
-        <v>2425</v>
+        <v>3636</v>
       </c>
       <c r="V3" t="n">
-        <v>6397</v>
+        <v>3921</v>
       </c>
       <c r="W3" t="n">
-        <v>3231</v>
+        <v>3375</v>
       </c>
       <c r="X3" t="n">
-        <v>21001</v>
+        <v>17851</v>
       </c>
       <c r="Y3" t="n">
-        <v>19434</v>
+        <v>35272</v>
       </c>
       <c r="Z3" t="n">
-        <v>-108.5</v>
+        <v>-299.64</v>
       </c>
       <c r="AA3" t="n">
-        <v>-31022</v>
+        <v>-16073</v>
       </c>
       <c r="AB3" t="n">
-        <v>-19613</v>
+        <v>-13852</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
       </c>
       <c r="AD3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -1800,94 +1800,94 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45836</v>
+        <v>45927</v>
       </c>
       <c r="B4" t="n">
-        <v>-33.54</v>
+        <v>37.27</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>-22.86</v>
+        <v>-11.45</v>
       </c>
       <c r="E4" t="n">
-        <v>-388</v>
+        <v>3441</v>
       </c>
       <c r="F4" t="n">
-        <v>-22.69</v>
+        <v>29.76</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>1.42</v>
       </c>
       <c r="H4" t="n">
-        <v>97865599.99999999</v>
+        <v>151444700</v>
       </c>
       <c r="I4" t="n">
-        <v>58534</v>
+        <v>57983</v>
       </c>
       <c r="J4" t="n">
-        <v>21206</v>
+        <v>19794</v>
       </c>
       <c r="K4" t="n">
-        <v>37328</v>
+        <v>38189</v>
       </c>
       <c r="L4" t="n">
-        <v>-9.74</v>
+        <v>-60.43</v>
       </c>
       <c r="M4" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="N4" t="n">
-        <v>-35.26</v>
+        <v>-300.05</v>
       </c>
       <c r="O4" t="n">
-        <v>-22.46</v>
+        <v>-15.34</v>
       </c>
       <c r="P4" t="n">
-        <v>-14.45</v>
+        <v>-12.54</v>
       </c>
       <c r="Q4" t="n">
-        <v>2050</v>
+        <v>2546</v>
       </c>
       <c r="R4" t="n">
-        <v>-2086</v>
+        <v>-6250</v>
       </c>
       <c r="S4" t="n">
-        <v>782</v>
+        <v>5152</v>
       </c>
       <c r="T4" t="n">
-        <v>-1500</v>
+        <v>121</v>
       </c>
       <c r="U4" t="n">
-        <v>3550</v>
+        <v>2425</v>
       </c>
       <c r="V4" t="n">
-        <v>10209</v>
+        <v>6397</v>
       </c>
       <c r="W4" t="n">
-        <v>3684</v>
+        <v>3231</v>
       </c>
       <c r="X4" t="n">
-        <v>25821</v>
+        <v>21001</v>
       </c>
       <c r="Y4" t="n">
-        <v>8409</v>
+        <v>19434</v>
       </c>
       <c r="Z4" t="n">
-        <v>-110.02</v>
+        <v>-108.5</v>
       </c>
       <c r="AA4" t="n">
-        <v>-33395</v>
+        <v>-31022</v>
       </c>
       <c r="AB4" t="n">
-        <v>-25094</v>
+        <v>-19613</v>
       </c>
       <c r="AC4" t="n">
         <v>0</v>
       </c>
       <c r="AD4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
@@ -1895,88 +1895,88 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45745</v>
+        <v>45836</v>
       </c>
       <c r="B5" t="n">
-        <v>-120.13</v>
+        <v>-33.54</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>-19.99</v>
+        <v>-22.86</v>
       </c>
       <c r="E5" t="n">
-        <v>2124</v>
+        <v>-388</v>
       </c>
       <c r="F5" t="n">
-        <v>-6.48</v>
+        <v>-22.69</v>
       </c>
       <c r="G5" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>98629530</v>
+        <v>97865599.99999999</v>
       </c>
       <c r="I5" t="n">
-        <v>58895</v>
+        <v>58534</v>
       </c>
       <c r="J5" t="n">
-        <v>21048</v>
+        <v>21206</v>
       </c>
       <c r="K5" t="n">
-        <v>37847</v>
+        <v>37328</v>
       </c>
       <c r="L5" t="n">
-        <v>-16.35</v>
+        <v>-9.74</v>
       </c>
       <c r="M5" t="n">
         <v>0.38</v>
       </c>
       <c r="N5" t="n">
-        <v>-58.95</v>
+        <v>-35.26</v>
       </c>
       <c r="O5" t="n">
-        <v>-19.5</v>
+        <v>-22.46</v>
       </c>
       <c r="P5" t="n">
-        <v>-12.58</v>
+        <v>-14.45</v>
       </c>
       <c r="Q5" t="n">
-        <v>813</v>
+        <v>2050</v>
       </c>
       <c r="R5" t="n">
-        <v>81</v>
+        <v>-2086</v>
       </c>
       <c r="S5" t="n">
-        <v>-196</v>
+        <v>782</v>
       </c>
       <c r="T5" t="n">
-        <v>-4370</v>
+        <v>-1500</v>
       </c>
       <c r="U5" t="n">
-        <v>5183</v>
+        <v>3550</v>
       </c>
       <c r="V5" t="n">
-        <v>13217</v>
+        <v>10209</v>
       </c>
       <c r="W5" t="n">
-        <v>3640</v>
+        <v>3684</v>
       </c>
       <c r="X5" t="n">
-        <v>29527</v>
+        <v>25821</v>
       </c>
       <c r="Y5" t="n">
-        <v>9960</v>
+        <v>8409</v>
       </c>
       <c r="Z5" t="n">
-        <v>-156.87</v>
+        <v>-110.02</v>
       </c>
       <c r="AA5" t="n">
-        <v>-33774</v>
+        <v>-33395</v>
       </c>
       <c r="AB5" t="n">
-        <v>-33762</v>
+        <v>-25094</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
@@ -1990,94 +1990,94 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45563</v>
+        <v>45745</v>
       </c>
       <c r="B6" t="n">
-        <v>-6.05</v>
+        <v>-120.13</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>-18.24</v>
+        <v>-19.99</v>
       </c>
       <c r="E6" t="n">
-        <v>-5809</v>
+        <v>2124</v>
       </c>
       <c r="F6" t="n">
-        <v>-125.26</v>
+        <v>-6.48</v>
       </c>
       <c r="G6" t="n">
-        <v>1.01</v>
+        <v>0.99</v>
       </c>
       <c r="H6" t="n">
-        <v>100690320</v>
+        <v>98629530</v>
       </c>
       <c r="I6" t="n">
-        <v>57284</v>
+        <v>58895</v>
       </c>
       <c r="J6" t="n">
-        <v>24086</v>
+        <v>21048</v>
       </c>
       <c r="K6" t="n">
-        <v>33198</v>
+        <v>37847</v>
       </c>
       <c r="L6" t="n">
-        <v>-13.68</v>
+        <v>-16.35</v>
       </c>
       <c r="M6" t="n">
-        <v>0.33</v>
+        <v>0.38</v>
       </c>
       <c r="N6" t="n">
-        <v>-55.17</v>
+        <v>-58.95</v>
       </c>
       <c r="O6" t="n">
-        <v>-18.42</v>
+        <v>-19.5</v>
       </c>
       <c r="P6" t="n">
-        <v>-12.12</v>
+        <v>-12.58</v>
       </c>
       <c r="Q6" t="n">
-        <v>4054</v>
+        <v>813</v>
       </c>
       <c r="R6" t="n">
-        <v>-2764</v>
+        <v>81</v>
       </c>
       <c r="S6" t="n">
-        <v>-3792</v>
+        <v>-196</v>
       </c>
       <c r="T6" t="n">
-        <v>-2404</v>
+        <v>-4370</v>
       </c>
       <c r="U6" t="n">
-        <v>6458</v>
+        <v>5183</v>
       </c>
       <c r="V6" t="n">
-        <v>14192</v>
+        <v>13217</v>
       </c>
       <c r="W6" t="n">
-        <v>4049</v>
+        <v>3640</v>
       </c>
       <c r="X6" t="n">
-        <v>30732</v>
+        <v>29527</v>
       </c>
       <c r="Y6" t="n">
-        <v>10978</v>
+        <v>9960</v>
       </c>
       <c r="Z6" t="n">
-        <v>-132.86</v>
+        <v>-156.87</v>
       </c>
       <c r="AA6" t="n">
-        <v>-26359</v>
+        <v>-33774</v>
       </c>
       <c r="AB6" t="n">
-        <v>-31334</v>
+        <v>-33762</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>-3.22</v>
+        <v>-0</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
@@ -2085,94 +2085,94 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45472</v>
+        <v>45563</v>
       </c>
       <c r="B7" t="n">
-        <v>-81.55</v>
+        <v>-6.05</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.16</v>
+        <v>-18.24</v>
       </c>
       <c r="E7" t="n">
-        <v>239</v>
+        <v>-5809</v>
       </c>
       <c r="F7" t="n">
-        <v>-12.55</v>
+        <v>-125.26</v>
       </c>
       <c r="G7" t="n">
-        <v>1.14</v>
+        <v>1.01</v>
       </c>
       <c r="H7" t="n">
-        <v>131295590</v>
+        <v>100690320</v>
       </c>
       <c r="I7" t="n">
-        <v>58439</v>
+        <v>57284</v>
       </c>
       <c r="J7" t="n">
-        <v>29273</v>
+        <v>24086</v>
       </c>
       <c r="K7" t="n">
-        <v>29166</v>
+        <v>33198</v>
       </c>
       <c r="L7" t="n">
-        <v>6.95</v>
+        <v>-13.68</v>
       </c>
       <c r="M7" t="n">
-        <v>0.25</v>
+        <v>0.33</v>
       </c>
       <c r="N7" t="n">
-        <v>38.22</v>
+        <v>-55.17</v>
       </c>
       <c r="O7" t="n">
-        <v>-0.18</v>
+        <v>-18.42</v>
       </c>
       <c r="P7" t="n">
-        <v>-0.45</v>
+        <v>-12.12</v>
       </c>
       <c r="Q7" t="n">
-        <v>2292</v>
+        <v>4054</v>
       </c>
       <c r="R7" t="n">
-        <v>-9165</v>
+        <v>-2764</v>
       </c>
       <c r="S7" t="n">
-        <v>11237</v>
+        <v>-3792</v>
       </c>
       <c r="T7" t="n">
-        <v>-3390</v>
+        <v>-2404</v>
       </c>
       <c r="U7" t="n">
-        <v>5682</v>
+        <v>6458</v>
       </c>
       <c r="V7" t="n">
-        <v>15038</v>
+        <v>14192</v>
       </c>
       <c r="W7" t="n">
-        <v>4239</v>
+        <v>4049</v>
       </c>
       <c r="X7" t="n">
-        <v>31609</v>
+        <v>30732</v>
       </c>
       <c r="Y7" t="n">
-        <v>18802</v>
+        <v>10978</v>
       </c>
       <c r="Z7" t="n">
-        <v>-4144.570000000001</v>
+        <v>-132.86</v>
       </c>
       <c r="AA7" t="n">
-        <v>-12934</v>
+        <v>-26359</v>
       </c>
       <c r="AB7" t="n">
-        <v>-19565</v>
+        <v>-31334</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="AD7" t="n">
-        <v>-33.17</v>
+        <v>-3.22</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
@@ -2180,94 +2180,94 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45381</v>
+        <v>45472</v>
       </c>
       <c r="B8" t="n">
-        <v>-486.66</v>
+        <v>-81.55</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.75</v>
+        <v>-0.16</v>
       </c>
       <c r="E8" t="n">
-        <v>1131</v>
+        <v>239</v>
       </c>
       <c r="F8" t="n">
-        <v>-2.99</v>
+        <v>-12.55</v>
       </c>
       <c r="G8" t="n">
-        <v>1.75</v>
+        <v>1.14</v>
       </c>
       <c r="H8" t="n">
-        <v>185417820</v>
+        <v>131295590</v>
       </c>
       <c r="I8" t="n">
-        <v>59345</v>
+        <v>58439</v>
       </c>
       <c r="J8" t="n">
-        <v>21311</v>
+        <v>29273</v>
       </c>
       <c r="K8" t="n">
-        <v>38034</v>
+        <v>29166</v>
       </c>
       <c r="L8" t="n">
-        <v>8.66</v>
+        <v>6.95</v>
       </c>
       <c r="M8" t="n">
-        <v>0.36</v>
+        <v>0.25</v>
       </c>
       <c r="N8" t="n">
-        <v>50.88</v>
+        <v>38.22</v>
       </c>
       <c r="O8" t="n">
-        <v>-1.28</v>
+        <v>-0.18</v>
       </c>
       <c r="P8" t="n">
-        <v>-1.35</v>
+        <v>-0.45</v>
       </c>
       <c r="Q8" t="n">
-        <v>-1223</v>
+        <v>2292</v>
       </c>
       <c r="R8" t="n">
-        <v>-2563</v>
+        <v>-9165</v>
       </c>
       <c r="S8" t="n">
-        <v>3630</v>
+        <v>11237</v>
       </c>
       <c r="T8" t="n">
-        <v>-7193</v>
+        <v>-3390</v>
       </c>
       <c r="U8" t="n">
-        <v>5970</v>
+        <v>5682</v>
       </c>
       <c r="V8" t="n">
-        <v>17071</v>
+        <v>15038</v>
       </c>
       <c r="W8" t="n">
-        <v>4382</v>
+        <v>4239</v>
       </c>
       <c r="X8" t="n">
-        <v>33512</v>
+        <v>31609</v>
       </c>
       <c r="Y8" t="n">
-        <v>15395</v>
+        <v>18802</v>
       </c>
       <c r="Z8" t="n">
-        <v>-1705.45</v>
+        <v>-4144.570000000001</v>
       </c>
       <c r="AA8" t="n">
-        <v>-12830</v>
+        <v>-12934</v>
       </c>
       <c r="AB8" t="n">
-        <v>-25288</v>
+        <v>-19565</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="AD8" t="n">
-        <v>-138.85</v>
+        <v>-33.17</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
@@ -2275,94 +2275,94 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45199</v>
+        <v>45381</v>
       </c>
       <c r="B9" t="n">
-        <v>494.76</v>
+        <v>-486.66</v>
       </c>
       <c r="C9" t="n">
-        <v>3497</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.03</v>
+        <v>-0.75</v>
       </c>
       <c r="E9" t="n">
-        <v>2012</v>
+        <v>1131</v>
       </c>
       <c r="F9" t="n">
-        <v>2.1</v>
+        <v>-2.99</v>
       </c>
       <c r="G9" t="n">
-        <v>1.44</v>
+        <v>1.75</v>
       </c>
       <c r="H9" t="n">
-        <v>146943940</v>
+        <v>185417820</v>
       </c>
       <c r="I9" t="n">
-        <v>56825</v>
+        <v>59345</v>
       </c>
       <c r="J9" t="n">
-        <v>25030</v>
+        <v>21311</v>
       </c>
       <c r="K9" t="n">
-        <v>31795</v>
+        <v>38034</v>
       </c>
       <c r="L9" t="n">
-        <v>5.42</v>
+        <v>8.66</v>
       </c>
       <c r="M9" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="N9" t="n">
-        <v>30.47</v>
+        <v>50.88</v>
       </c>
       <c r="O9" t="n">
-        <v>0.04</v>
+        <v>-1.28</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.26</v>
+        <v>-1.35</v>
       </c>
       <c r="Q9" t="n">
-        <v>5824</v>
+        <v>-1223</v>
       </c>
       <c r="R9" t="n">
-        <v>-7394</v>
+        <v>-2563</v>
       </c>
       <c r="S9" t="n">
-        <v>842</v>
+        <v>3630</v>
       </c>
       <c r="T9" t="n">
-        <v>71</v>
+        <v>-7193</v>
       </c>
       <c r="U9" t="n">
-        <v>5753</v>
+        <v>5970</v>
       </c>
       <c r="V9" t="n">
-        <v>17819</v>
+        <v>17071</v>
       </c>
       <c r="W9" t="n">
-        <v>3870</v>
+        <v>4382</v>
       </c>
       <c r="X9" t="n">
-        <v>34180</v>
+        <v>33512</v>
       </c>
       <c r="Y9" t="n">
-        <v>15197</v>
+        <v>15395</v>
       </c>
       <c r="Z9" t="n">
-        <v>-7766.35</v>
+        <v>-1705.45</v>
       </c>
       <c r="AA9" t="n">
-        <v>-4552</v>
+        <v>-12830</v>
       </c>
       <c r="AB9" t="n">
-        <v>-18847</v>
+        <v>-25288</v>
       </c>
       <c r="AC9" t="n">
         <v>0.12</v>
       </c>
       <c r="AD9" t="n">
-        <v>176.77</v>
+        <v>-138.85</v>
       </c>
       <c r="AE9" t="n">
         <v>0</v>
@@ -2370,94 +2370,94 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45078</v>
+        <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>92.53</v>
+        <v>494.76</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>3497</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.52</v>
+        <v>0.03</v>
       </c>
       <c r="E10" t="n">
-        <v>816</v>
+        <v>2012</v>
       </c>
       <c r="F10" t="n">
-        <v>11.44</v>
+        <v>2.1</v>
       </c>
       <c r="G10" t="n">
-        <v>1.36</v>
+        <v>1.44</v>
       </c>
       <c r="H10" t="n">
-        <v>137044140</v>
+        <v>146943940</v>
       </c>
       <c r="I10" t="n">
-        <v>56689</v>
+        <v>56825</v>
       </c>
       <c r="J10" t="n">
-        <v>24257</v>
+        <v>25030</v>
       </c>
       <c r="K10" t="n">
-        <v>32432</v>
+        <v>31795</v>
       </c>
       <c r="L10" t="n">
-        <v>5.56</v>
+        <v>5.42</v>
       </c>
       <c r="M10" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="N10" t="n">
-        <v>29.04</v>
+        <v>30.47</v>
       </c>
       <c r="O10" t="n">
-        <v>-0.7</v>
+        <v>0.04</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.65</v>
+        <v>-0.26</v>
       </c>
       <c r="Q10" t="n">
-        <v>2808</v>
+        <v>5824</v>
       </c>
       <c r="R10" t="n">
-        <v>-2808</v>
+        <v>-7394</v>
       </c>
       <c r="S10" t="n">
-        <v>117</v>
+        <v>842</v>
       </c>
       <c r="T10" t="n">
-        <v>-3080</v>
+        <v>71</v>
       </c>
       <c r="U10" t="n">
-        <v>5888</v>
+        <v>5753</v>
       </c>
       <c r="V10" t="n">
-        <v>18647</v>
+        <v>17819</v>
       </c>
       <c r="W10" t="n">
-        <v>4080</v>
+        <v>3870</v>
       </c>
       <c r="X10" t="n">
-        <v>35538</v>
+        <v>34180</v>
       </c>
       <c r="Y10" t="n">
-        <v>16176</v>
+        <v>15197</v>
       </c>
       <c r="Z10" t="n">
-        <v>-3695.68</v>
+        <v>-7766.35</v>
       </c>
       <c r="AA10" t="n">
-        <v>-11542</v>
+        <v>-4552</v>
       </c>
       <c r="AB10" t="n">
-        <v>-24090</v>
+        <v>-18847</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="AD10" t="n">
-        <v>35.38</v>
+        <v>176.77</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -2465,94 +2465,94 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>44986</v>
+        <v>45078</v>
       </c>
       <c r="B11" t="n">
-        <v>-48.03</v>
+        <v>92.53</v>
       </c>
       <c r="C11" t="n">
-        <v>21.69</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>4.61</v>
+        <v>-0.52</v>
       </c>
       <c r="E11" t="n">
-        <v>433</v>
+        <v>816</v>
       </c>
       <c r="F11" t="n">
-        <v>-23.54</v>
+        <v>11.44</v>
       </c>
       <c r="G11" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="H11" t="n">
-        <v>132471060</v>
+        <v>137044140</v>
       </c>
       <c r="I11" t="n">
-        <v>55113</v>
+        <v>56689</v>
       </c>
       <c r="J11" t="n">
-        <v>27534</v>
+        <v>24257</v>
       </c>
       <c r="K11" t="n">
-        <v>27579</v>
+        <v>32432</v>
       </c>
       <c r="L11" t="n">
-        <v>2.26</v>
+        <v>5.56</v>
       </c>
       <c r="M11" t="n">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="N11" t="n">
-        <v>13.11</v>
+        <v>29.04</v>
       </c>
       <c r="O11" t="n">
-        <v>6.04</v>
+        <v>-0.7</v>
       </c>
       <c r="P11" t="n">
-        <v>0.33</v>
+        <v>-0.65</v>
       </c>
       <c r="Q11" t="n">
-        <v>-1785</v>
+        <v>2808</v>
       </c>
       <c r="R11" t="n">
-        <v>-8521</v>
+        <v>-2808</v>
       </c>
       <c r="S11" t="n">
-        <v>7394</v>
+        <v>117</v>
       </c>
       <c r="T11" t="n">
-        <v>-9198</v>
+        <v>-3080</v>
       </c>
       <c r="U11" t="n">
-        <v>7413</v>
+        <v>5888</v>
       </c>
       <c r="V11" t="n">
-        <v>16348</v>
+        <v>18647</v>
       </c>
       <c r="W11" t="n">
-        <v>4109</v>
+        <v>4080</v>
       </c>
       <c r="X11" t="n">
-        <v>33521</v>
+        <v>35538</v>
       </c>
       <c r="Y11" t="n">
-        <v>20921</v>
+        <v>16176</v>
       </c>
       <c r="Z11" t="n">
-        <v>7077.889999999999</v>
+        <v>-3695.68</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1741</v>
+        <v>-11542</v>
       </c>
       <c r="AB11" t="n">
-        <v>-16360</v>
+        <v>-24090</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.36</v>
+        <v>0.13</v>
       </c>
       <c r="AD11" t="n">
-        <v>-54.82</v>
+        <v>35.38</v>
       </c>
       <c r="AE11" t="n">
         <v>0</v>
@@ -2560,94 +2560,94 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44805</v>
+        <v>44986</v>
       </c>
       <c r="B12" t="n">
-        <v>99.09</v>
+        <v>-48.03</v>
       </c>
       <c r="C12" t="n">
-        <v>6.44</v>
+        <v>21.69</v>
       </c>
       <c r="D12" t="n">
-        <v>15.54</v>
+        <v>4.61</v>
       </c>
       <c r="E12" t="n">
-        <v>2606</v>
+        <v>433</v>
       </c>
       <c r="F12" t="n">
-        <v>6.64</v>
+        <v>-23.54</v>
       </c>
       <c r="G12" t="n">
-        <v>1.01</v>
+        <v>1.35</v>
       </c>
       <c r="H12" t="n">
-        <v>100973360</v>
+        <v>132471060</v>
       </c>
       <c r="I12" t="n">
-        <v>45283</v>
+        <v>55113</v>
       </c>
       <c r="J12" t="n">
-        <v>22559</v>
+        <v>27534</v>
       </c>
       <c r="K12" t="n">
-        <v>22724</v>
+        <v>27579</v>
       </c>
       <c r="L12" t="n">
-        <v>1.17</v>
+        <v>2.26</v>
       </c>
       <c r="M12" t="n">
-        <v>0.23</v>
+        <v>0.28</v>
       </c>
       <c r="N12" t="n">
-        <v>6.34</v>
+        <v>13.11</v>
       </c>
       <c r="O12" t="n">
-        <v>15.52</v>
+        <v>6.04</v>
       </c>
       <c r="P12" t="n">
-        <v>6.04</v>
+        <v>0.33</v>
       </c>
       <c r="Q12" t="n">
-        <v>1030</v>
+        <v>-1785</v>
       </c>
       <c r="R12" t="n">
-        <v>-4574</v>
+        <v>-8521</v>
       </c>
       <c r="S12" t="n">
-        <v>3683</v>
+        <v>7394</v>
       </c>
       <c r="T12" t="n">
-        <v>-6269</v>
+        <v>-9198</v>
       </c>
       <c r="U12" t="n">
-        <v>7299</v>
+        <v>7413</v>
       </c>
       <c r="V12" t="n">
-        <v>12346</v>
+        <v>16348</v>
       </c>
       <c r="W12" t="n">
-        <v>4302</v>
+        <v>4109</v>
       </c>
       <c r="X12" t="n">
-        <v>29213</v>
+        <v>33521</v>
       </c>
       <c r="Y12" t="n">
-        <v>21450</v>
+        <v>20921</v>
       </c>
       <c r="Z12" t="n">
-        <v>387.53</v>
+        <v>7077.889999999999</v>
       </c>
       <c r="AA12" t="n">
-        <v>6022</v>
+        <v>-1741</v>
       </c>
       <c r="AB12" t="n">
-        <v>-64245</v>
+        <v>-16360</v>
       </c>
       <c r="AC12" t="n">
         <v>0.36</v>
       </c>
       <c r="AD12" t="n">
-        <v>147.4</v>
+        <v>-54.82</v>
       </c>
       <c r="AE12" t="n">
         <v>0</v>
@@ -2655,94 +2655,94 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44714</v>
+        <v>44805</v>
       </c>
       <c r="B13" t="n">
-        <v>-318.25</v>
+        <v>99.09</v>
       </c>
       <c r="C13" t="n">
-        <v>7.33</v>
+        <v>6.44</v>
       </c>
       <c r="D13" t="n">
-        <v>13.65</v>
+        <v>15.54</v>
       </c>
       <c r="E13" t="n">
-        <v>1981</v>
+        <v>2606</v>
       </c>
       <c r="F13" t="n">
-        <v>-2.96</v>
+        <v>6.64</v>
       </c>
       <c r="G13" t="n">
-        <v>1.43</v>
+        <v>1.01</v>
       </c>
       <c r="H13" t="n">
-        <v>144484000</v>
+        <v>100973360</v>
       </c>
       <c r="I13" t="n">
-        <v>40608</v>
+        <v>45283</v>
       </c>
       <c r="J13" t="n">
-        <v>27044</v>
+        <v>22559</v>
       </c>
       <c r="K13" t="n">
-        <v>13564</v>
+        <v>22724</v>
       </c>
       <c r="L13" t="n">
-        <v>0.55</v>
+        <v>1.17</v>
       </c>
       <c r="M13" t="n">
-        <v>0.13</v>
+        <v>0.23</v>
       </c>
       <c r="N13" t="n">
-        <v>6.36</v>
+        <v>6.34</v>
       </c>
       <c r="O13" t="n">
-        <v>19.31</v>
+        <v>15.52</v>
       </c>
       <c r="P13" t="n">
-        <v>8.890000000000001</v>
+        <v>6.04</v>
       </c>
       <c r="Q13" t="n">
-        <v>809</v>
+        <v>1030</v>
       </c>
       <c r="R13" t="n">
-        <v>168</v>
+        <v>-4574</v>
       </c>
       <c r="S13" t="n">
-        <v>-2802</v>
+        <v>3683</v>
       </c>
       <c r="T13" t="n">
-        <v>-6433</v>
+        <v>-6269</v>
       </c>
       <c r="U13" t="n">
-        <v>7242</v>
+        <v>7299</v>
       </c>
       <c r="V13" t="n">
-        <v>9022</v>
+        <v>12346</v>
       </c>
       <c r="W13" t="n">
-        <v>4400</v>
+        <v>4302</v>
       </c>
       <c r="X13" t="n">
-        <v>25302</v>
+        <v>29213</v>
       </c>
       <c r="Y13" t="n">
-        <v>23370</v>
+        <v>21450</v>
       </c>
       <c r="Z13" t="n">
-        <v>224.4</v>
+        <v>387.53</v>
       </c>
       <c r="AA13" t="n">
-        <v>10031</v>
+        <v>6022</v>
       </c>
       <c r="AB13" t="n">
-        <v>-4800</v>
+        <v>-64245</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="AD13" t="n">
-        <v>-330.18</v>
+        <v>147.4</v>
       </c>
       <c r="AE13" t="n">
         <v>0</v>
@@ -2750,94 +2750,94 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44622</v>
+        <v>44714</v>
       </c>
       <c r="B14" t="n">
-        <v>23.29</v>
+        <v>-318.25</v>
       </c>
       <c r="C14" t="n">
-        <v>8.06</v>
+        <v>7.33</v>
       </c>
       <c r="D14" t="n">
-        <v>12.41</v>
+        <v>13.65</v>
       </c>
       <c r="E14" t="n">
-        <v>7188</v>
+        <v>1981</v>
       </c>
       <c r="F14" t="n">
-        <v>44.21</v>
+        <v>-2.96</v>
       </c>
       <c r="G14" t="n">
-        <v>1.83</v>
+        <v>1.43</v>
       </c>
       <c r="H14" t="n">
-        <v>188939280</v>
+        <v>144484000</v>
       </c>
       <c r="I14" t="n">
-        <v>42438</v>
+        <v>40608</v>
       </c>
       <c r="J14" t="n">
-        <v>38696</v>
+        <v>27044</v>
       </c>
       <c r="K14" t="n">
-        <v>3742</v>
+        <v>13564</v>
       </c>
       <c r="L14" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M14" t="n">
         <v>0.13</v>
       </c>
-      <c r="M14" t="n">
-        <v>0.04</v>
-      </c>
       <c r="N14" t="n">
-        <v>6.64</v>
+        <v>6.36</v>
       </c>
       <c r="O14" t="n">
-        <v>22.65</v>
+        <v>19.31</v>
       </c>
       <c r="P14" t="n">
-        <v>10.99</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="Q14" t="n">
-        <v>5891</v>
+        <v>809</v>
       </c>
       <c r="R14" t="n">
-        <v>-2640</v>
+        <v>168</v>
       </c>
       <c r="S14" t="n">
-        <v>-1863</v>
+        <v>-2802</v>
       </c>
       <c r="T14" t="n">
-        <v>1287</v>
+        <v>-6433</v>
       </c>
       <c r="U14" t="n">
-        <v>4604</v>
+        <v>7242</v>
       </c>
       <c r="V14" t="n">
-        <v>5979</v>
+        <v>9022</v>
       </c>
       <c r="W14" t="n">
-        <v>4362</v>
+        <v>4400</v>
       </c>
       <c r="X14" t="n">
-        <v>21482</v>
+        <v>25302</v>
       </c>
       <c r="Y14" t="n">
-        <v>33246</v>
+        <v>23370</v>
       </c>
       <c r="Z14" t="n">
-        <v>139.6</v>
+        <v>224.4</v>
       </c>
       <c r="AA14" t="n">
-        <v>20706</v>
+        <v>10031</v>
       </c>
       <c r="AB14" t="n">
-        <v>8967</v>
+        <v>-4800</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="AD14" t="n">
-        <v>18.33</v>
+        <v>-330.18</v>
       </c>
       <c r="AE14" t="n">
         <v>0</v>
@@ -2845,94 +2845,94 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44464</v>
+        <v>44622</v>
       </c>
       <c r="B15" t="n">
-        <v>29.21</v>
+        <v>23.29</v>
       </c>
       <c r="C15" t="n">
-        <v>10.27</v>
+        <v>8.06</v>
       </c>
       <c r="D15" t="n">
-        <v>9.74</v>
+        <v>12.41</v>
       </c>
       <c r="E15" t="n">
-        <v>7722</v>
+        <v>7188</v>
       </c>
       <c r="F15" t="n">
-        <v>35.55</v>
+        <v>44.21</v>
       </c>
       <c r="G15" t="n">
-        <v>2.21</v>
+        <v>1.83</v>
       </c>
       <c r="H15" t="n">
-        <v>199273270</v>
+        <v>188939280</v>
       </c>
       <c r="I15" t="n">
-        <v>45693</v>
+        <v>42438</v>
       </c>
       <c r="J15" t="n">
-        <v>11874</v>
+        <v>38696</v>
       </c>
       <c r="K15" t="n">
-        <v>33819</v>
+        <v>3742</v>
       </c>
       <c r="L15" t="n">
-        <v>1.14</v>
+        <v>0.13</v>
       </c>
       <c r="M15" t="n">
-        <v>0.38</v>
+        <v>0.04</v>
       </c>
       <c r="N15" t="n">
-        <v>7.89</v>
+        <v>6.64</v>
       </c>
       <c r="O15" t="n">
-        <v>21.67</v>
+        <v>22.65</v>
       </c>
       <c r="P15" t="n">
-        <v>12.89</v>
+        <v>10.99</v>
       </c>
       <c r="Q15" t="n">
-        <v>9900</v>
+        <v>5891</v>
       </c>
       <c r="R15" t="n">
-        <v>-10682</v>
+        <v>-2640</v>
       </c>
       <c r="S15" t="n">
-        <v>3906</v>
+        <v>-1863</v>
       </c>
       <c r="T15" t="n">
-        <v>5895</v>
+        <v>1287</v>
       </c>
       <c r="U15" t="n">
-        <v>4005</v>
+        <v>4604</v>
       </c>
       <c r="V15" t="n">
-        <v>5261</v>
+        <v>5979</v>
       </c>
       <c r="W15" t="n">
-        <v>3803</v>
+        <v>4362</v>
       </c>
       <c r="X15" t="n">
-        <v>19674</v>
+        <v>21482</v>
       </c>
       <c r="Y15" t="n">
-        <v>31732</v>
+        <v>33246</v>
       </c>
       <c r="Z15" t="n">
-        <v>111.92</v>
+        <v>139.6</v>
       </c>
       <c r="AA15" t="n">
-        <v>17075</v>
+        <v>20706</v>
       </c>
       <c r="AB15" t="n">
-        <v>14256</v>
+        <v>8967</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="AD15" t="n">
-        <v>20.67</v>
+        <v>18.33</v>
       </c>
       <c r="AE15" t="n">
         <v>0</v>
@@ -2940,191 +2940,286 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44373</v>
+        <v>44464</v>
       </c>
       <c r="B16" t="n">
-        <v>41.1</v>
+        <v>29.21</v>
       </c>
       <c r="C16" t="n">
-        <v>11.95</v>
+        <v>10.27</v>
       </c>
       <c r="D16" t="n">
-        <v>8.369999999999999</v>
+        <v>9.74</v>
       </c>
       <c r="E16" t="n">
-        <v>7954</v>
+        <v>7722</v>
       </c>
       <c r="F16" t="n">
-        <v>25.78</v>
+        <v>35.55</v>
       </c>
       <c r="G16" t="n">
-        <v>2.44</v>
+        <v>2.21</v>
       </c>
       <c r="H16" t="n">
-        <v>207997130</v>
+        <v>199273270</v>
       </c>
       <c r="I16" t="n">
-        <v>40738</v>
+        <v>45693</v>
       </c>
       <c r="J16" t="n">
-        <v>7760</v>
+        <v>11874</v>
       </c>
       <c r="K16" t="n">
-        <v>32978</v>
+        <v>33819</v>
       </c>
       <c r="L16" t="n">
-        <v>1.09</v>
+        <v>1.14</v>
       </c>
       <c r="M16" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="N16" t="n">
-        <v>7.99</v>
+        <v>7.89</v>
       </c>
       <c r="O16" t="n">
-        <v>20.89</v>
+        <v>21.67</v>
       </c>
       <c r="P16" t="n">
-        <v>13.63</v>
+        <v>12.89</v>
       </c>
       <c r="Q16" t="n">
-        <v>8746</v>
+        <v>9900</v>
       </c>
       <c r="R16" t="n">
-        <v>-6904</v>
+        <v>-10682</v>
       </c>
       <c r="S16" t="n">
-        <v>-2288</v>
+        <v>3906</v>
       </c>
       <c r="T16" t="n">
-        <v>5144</v>
+        <v>5895</v>
       </c>
       <c r="U16" t="n">
-        <v>3602</v>
+        <v>4005</v>
       </c>
       <c r="V16" t="n">
-        <v>4534</v>
+        <v>5261</v>
       </c>
       <c r="W16" t="n">
-        <v>3715</v>
+        <v>3803</v>
       </c>
       <c r="X16" t="n">
-        <v>18498</v>
+        <v>19674</v>
       </c>
       <c r="Y16" t="n">
-        <v>24536</v>
+        <v>31732</v>
       </c>
       <c r="Z16" t="n">
-        <v>107.03</v>
+        <v>111.92</v>
       </c>
       <c r="AA16" t="n">
-        <v>9438</v>
+        <v>17075</v>
       </c>
       <c r="AB16" t="n">
-        <v>13200</v>
+        <v>14256</v>
       </c>
       <c r="AC16" t="n">
         <v>0.35</v>
       </c>
       <c r="AD16" t="n">
-        <v>27.86</v>
+        <v>20.67</v>
       </c>
       <c r="AE16" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>44282</v>
+        <v>44373</v>
       </c>
       <c r="B17" t="n">
-        <v>70.25</v>
+        <v>41.1</v>
       </c>
       <c r="C17" t="n">
-        <v>13.29</v>
+        <v>11.95</v>
       </c>
       <c r="D17" t="n">
-        <v>7.52</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="E17" t="n">
-        <v>6148</v>
+        <v>7954</v>
       </c>
       <c r="F17" t="n">
-        <v>17.08</v>
+        <v>25.78</v>
       </c>
       <c r="G17" t="n">
-        <v>2.96</v>
+        <v>2.44</v>
       </c>
       <c r="H17" t="n">
-        <v>236099760</v>
+        <v>207997130</v>
       </c>
       <c r="I17" t="n">
-        <v>41206</v>
+        <v>40738</v>
       </c>
       <c r="J17" t="n">
-        <v>7609</v>
+        <v>7760</v>
       </c>
       <c r="K17" t="n">
-        <v>33597</v>
+        <v>32978</v>
       </c>
       <c r="L17" t="n">
-        <v>1.05</v>
+        <v>1.09</v>
       </c>
       <c r="M17" t="n">
-        <v>0.42</v>
+        <v>0.39</v>
       </c>
       <c r="N17" t="n">
-        <v>8.460000000000001</v>
+        <v>7.99</v>
       </c>
       <c r="O17" t="n">
-        <v>23.06</v>
+        <v>20.89</v>
       </c>
       <c r="P17" t="n">
-        <v>15.2</v>
+        <v>13.63</v>
       </c>
       <c r="Q17" t="n">
-        <v>5548</v>
+        <v>8746</v>
       </c>
       <c r="R17" t="n">
-        <v>-2547</v>
+        <v>-6904</v>
       </c>
       <c r="S17" t="n">
-        <v>-3674</v>
+        <v>-2288</v>
       </c>
       <c r="T17" t="n">
-        <v>1576</v>
+        <v>5144</v>
       </c>
       <c r="U17" t="n">
-        <v>3972</v>
+        <v>3602</v>
       </c>
       <c r="V17" t="n">
-        <v>3985</v>
+        <v>4534</v>
       </c>
       <c r="W17" t="n">
-        <v>3623</v>
+        <v>3715</v>
       </c>
       <c r="X17" t="n">
-        <v>17509</v>
+        <v>18498</v>
       </c>
       <c r="Y17" t="n">
-        <v>21622</v>
+        <v>24536</v>
       </c>
       <c r="Z17" t="n">
-        <v>111.76</v>
+        <v>107.03</v>
       </c>
       <c r="AA17" t="n">
-        <v>17090</v>
+        <v>9438</v>
       </c>
       <c r="AB17" t="n">
-        <v>11455</v>
+        <v>13200</v>
       </c>
       <c r="AC17" t="n">
         <v>0.35</v>
       </c>
       <c r="AD17" t="n">
+        <v>27.86</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>44282</v>
+      </c>
+      <c r="B18" t="n">
+        <v>70.25</v>
+      </c>
+      <c r="C18" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="E18" t="n">
+        <v>6148</v>
+      </c>
+      <c r="F18" t="n">
+        <v>17.08</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="H18" t="n">
+        <v>236099760</v>
+      </c>
+      <c r="I18" t="n">
+        <v>41206</v>
+      </c>
+      <c r="J18" t="n">
+        <v>7609</v>
+      </c>
+      <c r="K18" t="n">
+        <v>33597</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="N18" t="n">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="O18" t="n">
+        <v>23.06</v>
+      </c>
+      <c r="P18" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>5548</v>
+      </c>
+      <c r="R18" t="n">
+        <v>-2547</v>
+      </c>
+      <c r="S18" t="n">
+        <v>-3674</v>
+      </c>
+      <c r="T18" t="n">
+        <v>1576</v>
+      </c>
+      <c r="U18" t="n">
+        <v>3972</v>
+      </c>
+      <c r="V18" t="n">
+        <v>3985</v>
+      </c>
+      <c r="W18" t="n">
+        <v>3623</v>
+      </c>
+      <c r="X18" t="n">
+        <v>17509</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>21622</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>111.76</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>17090</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>11455</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AD18" t="n">
         <v>41.98</v>
       </c>
-      <c r="AE17" t="n">
+      <c r="AE18" t="n">
         <v>2301</v>
       </c>
     </row>

</xml_diff>